<commit_message>
test: use sequential fallback selectors for owner login button verification
</commit_message>
<xml_diff>
--- a/smart_press_selenium/reports/E2E_Web_Test_Report.xlsx
+++ b/smart_press_selenium/reports/E2E_Web_Test_Report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="57">
   <si>
     <t>Smart Press Web E2E Automation Test Summary</t>
   </si>
@@ -26,7 +26,7 @@
     <t>Date of Execution</t>
   </si>
   <si>
-    <t>13/6/2026 10:13:30 am</t>
+    <t>16/6/2026 7:56:20 pm</t>
   </si>
   <si>
     <t>Total Steps Executed</t>
@@ -62,7 +62,7 @@
     <t>Error / Failure Details</t>
   </si>
   <si>
-    <t>10:11:44 am</t>
+    <t>7:54:33 pm</t>
   </si>
   <si>
     <t>Smart Press Web - Authentication E2E Flow</t>
@@ -74,34 +74,34 @@
     <t>FAIL</t>
   </si>
   <si>
-    <t>16025ms</t>
+    <t>22402ms</t>
   </si>
   <si>
     <t>element ("[object Object]") still not displayed after 15000ms</t>
   </si>
   <si>
-    <t>10:11:54 am</t>
+    <t>7:54:43 pm</t>
   </si>
   <si>
     <t>should enter mobile number and request OTP</t>
   </si>
   <si>
-    <t>10043ms</t>
+    <t>10031ms</t>
   </si>
   <si>
     <t>element ("[object Object]") still not displayed after 10000ms</t>
   </si>
   <si>
-    <t>10:12:04 am</t>
+    <t>7:54:54 pm</t>
   </si>
   <si>
     <t>should read the development OTP and complete verification</t>
   </si>
   <si>
-    <t>10028ms</t>
-  </si>
-  <si>
-    <t>10:12:19 am</t>
+    <t>10045ms</t>
+  </si>
+  <si>
+    <t>7:55:09 pm</t>
   </si>
   <si>
     <t>Smart Press Web - Home Dashboard E2E Flow</t>
@@ -110,16 +110,13 @@
     <t>should verify metric cards are displayed properly</t>
   </si>
   <si>
-    <t>15046ms</t>
-  </si>
-  <si>
-    <t>10:12:20 am</t>
+    <t>15029ms</t>
   </si>
   <si>
     <t>should verify Today's Revenue section values</t>
   </si>
   <si>
-    <t>59ms</t>
+    <t>35ms</t>
   </si>
   <si>
     <t xml:space="preserve">expect(received).toBe(expected) // Object.is equality
@@ -130,10 +127,7 @@
     <t>should check all Quick Action buttons exist</t>
   </si>
   <si>
-    <t>43ms</t>
-  </si>
-  <si>
-    <t>10:12:35 am</t>
+    <t>7:55:24 pm</t>
   </si>
   <si>
     <t>Smart Press Web - Order Management E2E Flow</t>
@@ -145,25 +139,25 @@
     <t>15030ms</t>
   </si>
   <si>
-    <t>10:12:45 am</t>
+    <t>7:55:34 pm</t>
   </si>
   <si>
     <t>should configure order items and instructions</t>
   </si>
   <si>
-    <t>10036ms</t>
-  </si>
-  <si>
-    <t>Can't call click on element with selector "[object Object]" because element wasn't found</t>
-  </si>
-  <si>
-    <t>10:12:55 am</t>
+    <t>10107ms</t>
+  </si>
+  <si>
+    <t>7:55:44 pm</t>
   </si>
   <si>
     <t>should submit the order and check confirmation</t>
   </si>
   <si>
-    <t>10:13:10 am</t>
+    <t>10123ms</t>
+  </si>
+  <si>
+    <t>7:55:59 pm</t>
   </si>
   <si>
     <t>Smart Press Web - Reports &amp; Export E2E Flow</t>
@@ -172,25 +166,25 @@
     <t>should navigate to reports screen and verify sections</t>
   </si>
   <si>
-    <t>15045ms</t>
-  </si>
-  <si>
-    <t>10:13:20 am</t>
+    <t>15118ms</t>
+  </si>
+  <si>
+    <t>7:56:09 pm</t>
   </si>
   <si>
     <t>should navigate to export screen and select formats</t>
   </si>
   <si>
-    <t>10025ms</t>
-  </si>
-  <si>
-    <t>10:13:30 am</t>
+    <t>10168ms</t>
+  </si>
+  <si>
+    <t>7:56:20 pm</t>
   </si>
   <si>
     <t>should run export action and verify download start toast</t>
   </si>
   <si>
-    <t>10113ms</t>
+    <t>10371ms</t>
   </si>
 </sst>
 </file>
@@ -831,59 +825,59 @@
     </row>
     <row r="6" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>30</v>
       </c>
       <c r="C6" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="8" t="s">
+      <c r="F6" s="8" t="s">
         <v>35</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>30</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>19</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="D8" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>42</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>21</v>
@@ -891,59 +885,59 @@
     </row>
     <row r="9" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>45</v>
-      </c>
       <c r="F9" s="8" t="s">
-        <v>46</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>46</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="D11" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="8" t="s">
         <v>50</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>52</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>21</v>
@@ -951,42 +945,42 @@
     </row>
     <row r="12" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>55</v>
-      </c>
       <c r="F12" s="8" t="s">
-        <v>46</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>58</v>
-      </c>
       <c r="F13" s="8" t="s">
-        <v>46</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>